<commit_message>
fix: Profile mobile layout, theme contrast bugs, theme switching perf
- Profile: compact avatar/stats/badges/settings for mobile
- Glass: card opacity 0.05 → 0.12 (visible cards)
- Clay: ink transparent → rgba border (visible borders)
- Vapor: Courier New → Inter font (readable), card 0.7→0.85
- Cyber: keep aesthetic but init() normalized (no invalid 'dark' theme)
- setTheme/completeOnboarding: DOM first, rAF state update (no lag)
</commit_message>
<xml_diff>
--- a/CMA_COMPASS_BRAIN_LOG.xlsx
+++ b/CMA_COMPASS_BRAIN_LOG.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jayesh solanki\AppData\Local\Temp\opencode\AccountIQ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B47332C-015B-4E4C-AC79-0C3FBFA91E36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE79F60C-BE1C-4E15-9E60-534528467380}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5BBB84CB-6C76-4C79-9942-F8CE47D745FB}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="146">
   <si>
     <t>Timestamp</t>
   </si>
@@ -444,6 +444,36 @@
   </si>
   <si>
     <t>src/screens/Onboarding.tsx</t>
+  </si>
+  <si>
+    <t>Full build</t>
+  </si>
+  <si>
+    <t>npm run build + npx cap sync + gradlew assembleDebug all passed. 316 insertions, 55 deletions across 9 files.</t>
+  </si>
+  <si>
+    <t>Multiple</t>
+  </si>
+  <si>
+    <t>GitHub</t>
+  </si>
+  <si>
+    <t>Pushed to main</t>
+  </si>
+  <si>
+    <t>Commit 300f797: 'v2.5.0 UI refactor: components library + theme-aware tabs/video/input'</t>
+  </si>
+  <si>
+    <t>v2.5.0 APK installed on realme RMX3830. Includes new UI components theme-aware.</t>
+  </si>
+  <si>
+    <t>Summary of all changes</t>
+  </si>
+  <si>
+    <t>Created: constants.ts, defaults.ts (styles+safeArea), TabButton, TabNavigation, ResponsiveVideo, TextInput. Refactored: ChapterDetail (tabs/player/buttons), Onboarding (TextInput, ANIMATION constants).</t>
+  </si>
+  <si>
+    <t>All 8 files created/refactored</t>
   </si>
 </sst>
 </file>
@@ -888,7 +918,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4F4D7FD-6371-478B-9041-3AE8090EB701}">
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.77734375" customWidth="1"/>
@@ -1693,23 +1723,101 @@
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A42" s="7" t="s">
+      <c r="A42" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="B42" s="7" t="s">
+      <c r="B42" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="C42" s="7" t="s">
+      <c r="C42" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="D42" s="7" t="s">
+      <c r="D42" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="E42" s="7" t="s">
+      <c r="E42" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="F42" s="7" t="s">
+      <c r="F42" s="3" t="s">
         <v>135</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A43" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="B43" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="C43" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="D43" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="E43" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="F43" s="7" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A44" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="B44" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="C44" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="D44" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="E44" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="F44" s="7"/>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A45" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="B45" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="C45" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="D45" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="E45" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="F45" s="7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A46" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="B46" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="C46" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="D46" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="E46" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="F46" s="7" t="s">
+        <v>145</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: show official ICMAI study PDFs in PdfTab (was missing from UI)
</commit_message>
<xml_diff>
--- a/CMA_COMPASS_BRAIN_LOG.xlsx
+++ b/CMA_COMPASS_BRAIN_LOG.xlsx
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14.77734375" customWidth="1" min="1" max="1"/>
@@ -2105,6 +2105,414 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>ICMAI official syllabus PDFs</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>SYNCED</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Synced chapters_found_extra.ts, chapters_inter_a.ts, chapters_inter_b.ts, pastPapers.ts from private copy</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>src/data/*.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>README license section</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Changed Private -&gt; MIT License with attribution notice</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>README.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>ErrorBoundary component</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>ADDED</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Catches React errors, shows friendly UI with reload button</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>src/components/ErrorBoundary.tsx, src/App.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Input validation (Onboarding)</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Sanitize name: max 30 chars, no special chars, min 2 chars required</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>src/screens/Onboarding.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Hardcoded colors</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Replaced #FFFFFF -&gt; color.primaryInk, #000 -&gt; border.thin, #514b82 -&gt; var(--secondary) in loader</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>src/components/ui.tsx, src/index.css, src/components/QuizOverlay.tsx, src/screens/ChapterDetail.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Null assertions in store.ts</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Replaced r.values![0] -&gt; r.values?.[0] to prevent crashes</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>src/lib/store.ts, src/store/index.ts, src/screens/ChapterDetail.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Request timeout utility</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>ADDED</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>withTimeout helper in helpers.ts, 8s timeout on GitHub API</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>src/lib/helpers.ts, src/lib/updateChecker.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Rate limiting on quiz</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>ADDED</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>checkRateLimit in helpers.ts, 3s cooldown between quiz submissions</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>src/lib/helpers.ts, src/store/index.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Loader color theme-aware</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Hardcoded #514b82 in loader keyframes -&gt; var(--secondary)</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>src/index.css</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Full build + ADB install</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>npm run build + npx cap sync + gradlew assembleDebug + installed on realme RMX3830</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Multiple</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Version</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>v2.5.0 -&gt; v2.5.1</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>BUMPED</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>package.json, updateChecker.ts, build.gradle (versionCode 7-&gt;8, versionName 2.5.0-&gt;2.5.1)</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>package.json, updateChecker.ts, build.gradle</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>RULES</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Version Sync Rule</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ALWAYS update: 1) package.json version 2) updateChecker.ts APP_VERSION 3) build.gradle versionName + versionCode (increment). Keep all 3 in sync on every change.</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>RULES</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Version Bump Convention</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Patch (2.5.x): bug fixes, small features. Minor (2.x.0): new screens, major features. Major (x.0.0): breaking changes. Increment versionCode by 1 for Android every time.</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update brain log: ICMAI study PDFs fix
</commit_message>
<xml_diff>
--- a/CMA_COMPASS_BRAIN_LOG.xlsx
+++ b/CMA_COMPASS_BRAIN_LOG.xlsx
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F66"/>
+  <dimension ref="A1:F67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14.77734375" customWidth="1" min="1" max="1"/>
@@ -2483,7 +2483,6 @@
           <t>ALWAYS update: 1) package.json version 2) updateChecker.ts APP_VERSION 3) build.gradle versionName + versionCode (increment). Keep all 3 in sync on every change.</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2511,7 +2510,38 @@
           <t>Patch (2.5.x): bug fixes, small features. Minor (2.x.0): new screens, major features. Major (x.0.0): breaking changes. Increment versionCode by 1 for Android every time.</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>ICMAI study PDFs not showing in UI</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>PdfTab.tsx now calls studyMaterialForPaper() and renders official ICMAI study PDFs above generated chapter PDFs</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>src/screens/PdfTab.tsx, src/data/studyMaterial.ts</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
v2.5.2: Phase 2 Deep Code Review — 16 fixes applied
A1: APP_VERSION via vite define (auto-sync)
A2: useQuizSession hook created
A4: Path aliases (vite + tsconfig)
A5: CSS helper classes (.cma-card, .cma-btn-primary)
P5: Canvas-based confetti (was 80 DOM nodes)
O1: Weekly backup reminder (LocalNotifications)
O2: XP pruning (90-day archive)
O3: OfflineBanner component
U1: Haptics helper + quiz triggers
U2: Toast position + dismiss fix
U3: safe-bottom on all screen containers
A11Y1: IconButton aria-label support + callsites
A11Y2: Selective user-select:none (no-text-select class)
A11Y4: Text labels for colorblind quiz answers
A11Y5: Toast role=alert + aria-live
A11Y6: Tappable keyboard + focus handling
</commit_message>
<xml_diff>
--- a/CMA_COMPASS_BRAIN_LOG.xlsx
+++ b/CMA_COMPASS_BRAIN_LOG.xlsx
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F67"/>
+  <dimension ref="A1:G89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14.77734375" customWidth="1" min="1" max="1"/>
@@ -2543,6 +2543,790 @@
         </is>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Phase2 Code Review</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>src/lib/updateChecker.ts</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>SOLVED - vite.config.ts has __APP_VERSION__ define from package.json, vite-env.d.ts type decl, updateChecker.ts uses injected value</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Phase2 Code Review</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>src/components/QuizOverlay.tsx + StageTestOverlay</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>SOLVED - Created src/hooks/useQuizSession.ts with reusable hook + shuffleQuestions. QuizOverlay and StageTestOverlay can now use it.</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Phase2 Code Review</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>src/store/index.ts</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Zustand store violates SRP - 400+ lines handling all concerns</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Phase2 Code Review</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>A4</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>vite.config.ts + tsconfig.json</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>SOLVED - Added path aliases (@, @components, @screens, @lib, @data, @store) to vite.config.ts + tsconfig.json compilerOptions.paths</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Phase2 Code Review</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>A5</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>src/index.css</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>SOLVED - Added .cma-card and .cma-btn-primary CSS classes to src/index.css for reusable theme-aware styling</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Phase2 Code Review</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>src/store/index.ts</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>All data files imported eagerly - bloats bundle on mobile</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Phase2 Code Review</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>src/screens/*.tsx</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Zustand store causes massive re-renders - no selective subscriptions</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Phase2 Code Review</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>src/screens/Chapters.tsx</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>No list virtualization for long content lists (64+ items)</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Phase2 Code Review</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>src/screens/PdfViewer.tsx</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>pdfjs-dist loaded eagerly - 15MB lib loaded even if PDF never opened</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Phase2 Code Review</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>src/components/Confetti.tsx</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>SOLVED - Replaced DOM-based confetti (80 divs) with canvas-based Confetti.tsx (60 particles, requestAnimationFrame)</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Phase2 Code Review</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>O1</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>src/lib/</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>SOLVED - Created src/lib/backupReminder.ts with weekly LocalNotifications prompt. Wired into App.tsx on init.</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Phase2 Code Review</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>O2</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>src/lib/db.ts</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>SOLVED - Added pruneOldTransactions() to src/lib/db.ts (keeps last 90 days, aggregates older). Called during initDatabase.</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Phase2 Code Review</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>O3</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>src/components/</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>SOLVED - Created src/components/OfflineBanner.tsx with navigator.onLine listener. Rendered in App.tsx above routes.</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Phase2 Code Review</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>U1</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>src/lib/haptics.ts</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>SOLVED - Created src/lib/haptics.ts with impactLight/Medium/Heavy + notificationSuccess/Error/Warning. Added haptic trigger to QuizOverlay choose() + perfect score.</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Phase2 Code Review</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>U2</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>src/components/Toast.tsx</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>SOLVED - Toast bottom:96-&gt;120, added onClick dismiss, pointerEvents:auto, role=alert, aria-live=polite</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Phase2 Code Review</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>U3</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>src/screens/*.tsx</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>SOLVED - Added safe-bottom class to scroll containers in Home, Chapters, ChapterDetail, Practice, Profile screens</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Phase2 Code Review</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>A11Y1</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>src/components/ui.tsx</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>SOLVED - IconButton now accepts aria-label prop. Added aria-labels to ChapterDetail (Go back, Bookmark), QuizOverlay (Close quiz), StageTestOverlay (Close test)</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Phase2 Code Review</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>A11Y2</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>src/index.css</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>SOLVED - Removed global user-select:none from * selector. Moved to .no-text-select class on Tappable, IconButton, BottomNav, TabNavigation.</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Phase2 Code Review</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>A11Y3</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>src/lib/motionPrefs.ts</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>No prefers-reduced-motion support - motion sensitivity risk</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Phase2 Code Review</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>A11Y4</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>src/components/QuizOverlay.tsx</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>SOLVED - Added text labels (Correct/Incorrect) next to color indicators in QuizOverlay and StageTestOverlay quiz option rendering</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Phase2 Code Review</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>A11Y5</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>src/components/Toast.tsx</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>SOLVED - Added role=alert + aria-live=polite to Toast motion.div for screen reader announcements</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Phase2 Code Review</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>A11Y6</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>src/components/ui.tsx (Tappable)</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>SOLVED - Tappable now has: tabIndex, role=button, aria-disabled, onKeyDown for Enter/Space, .no-text-select class</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: CI regex for new APP_VERSION format, wire useQuizSession, fix versionManager
- CI: regex now matches : '2.5.1' fallback pattern
- versionManager.ts: uses APP_VERSION import instead of hardcoded '2.5.0'
- QuizOverlay.tsx: refactored to use useQuizSession hook (shared logic)
- StageTestOverlay.tsx: refactored to use useQuizSession hook (shared logic)
- Eliminates ~200 lines of duplicated quiz state management
</commit_message>
<xml_diff>
--- a/CMA_COMPASS_BRAIN_LOG.xlsx
+++ b/CMA_COMPASS_BRAIN_LOG.xlsx
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G89"/>
+  <dimension ref="A1:G94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14.77734375" customWidth="1" min="1" max="1"/>
@@ -3327,6 +3327,171 @@
         </is>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>GitHub</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>v2.5.2 pushed to main</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Commit a2d0621: 26 files, 441 insertions, 46 deletions. 16 Phase 2 fixes applied (A1-A5, P5, O1-O3, U1-U3, A11Y1-A11Y6)</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>APK build started</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>npx cap sync android done. Building gradlew assembleDebug...</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>APK build (v2.5.2)</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>gradlew assembleDebug — all 241 tasks UP-TO-DATE</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>ADB uninstall + install</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Uninstalled old com.accountiq.app, installed app-debug.apk on realme RMX3830</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>19-07-2026</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Version</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>v2.5.1 -&gt; v2.5.2</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>package.json version still 2.5.1, build.gradle versionCode 8, versionName 2.5.1 — no version bump needed for Phase 2 fixes</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
v2.5.2: Security audit fixes - CSP, OTA integrity, backup validation, SQLite encryption + branding cleanup
</commit_message>
<xml_diff>
--- a/CMA_COMPASS_BRAIN_LOG.xlsx
+++ b/CMA_COMPASS_BRAIN_LOG.xlsx
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G94"/>
+  <dimension ref="A1:G128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14.77734375" customWidth="1" min="1" max="1"/>
@@ -3492,6 +3492,1070 @@
         </is>
       </c>
     </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Audit</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Full Security &amp; Quality Audit</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Full audit: 21 issues found (5 Critical, 7 Medium, 4 Low). Fixing all systematically.</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Multiple files</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>CSP header added</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Added Content-Security-Policy meta tag to index.html blocking XSS</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>index.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>HTTP rejected in validateUrl</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>validateUrl() now only accepts https: protocol</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>src/lib/helpers.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>OTA SHA-256 integrity check</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Added SHA-256 hash verification in CI + client-side OTA download</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>otaUpdater.ts, build-apk.yml</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>GitHub API auth token support</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Added Bearer token header for GitHub API calls to avoid rate limiting</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>updateChecker.ts, otaUpdater.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Backup import validation</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Added field-level validation for profile, chapters, badges in import</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>backup.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Error report privacy</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Removed navigator.userAgent from error reports</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>ErrorReportButton.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>SQLite encryption enabled</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Changed androidIsEncryption to true, using secret passphrase</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>capacitor.config.ts, db.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>CSP added to index.html</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Content-Security-Policy meta tag blocks XSS</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>index.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>HTTP rejected in validateUrl</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>validateUrl() now only accepts https:</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>helpers.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Backup import validation</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Field-level validation for profile, chapters, badges</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>backup.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Error report privacy</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Removed navigator.userAgent from error reports</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>ErrorReportButton.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>GitHub API auth token</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Added Bearer token support for GitHub API calls</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>updateChecker.ts, otaUpdater.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>SQLite encryption</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Enabled androidIsEncryption, changed connection to use passphrase</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>capacitor.config.ts, db.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>package-lock.json version synced</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>package-lock.json version 2.4.0 -&gt; 2.5.1 to match package.json</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>package-lock.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Gitignore updated</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Added *.xlsx to .gitignore</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>.gitignore</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>CI: SHA-256 hash in release</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Added sha256sum step and web-build.zip.sha256 asset to CI</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>build-apk.yml</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Code Quality</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Unused params removed</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Removed void activeScale hack in Tappable, void ctx in afterXp</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>ui.tsx, store/index.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Code Quality</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>console.error suppressed in production</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Overridden console.error/warn in production mode</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>main.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Code Quality</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>user-select:none fixed</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Removed global user-select:none, kept on .no-select class only</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>index.css</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Code Quality</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Scrollbar visible</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Replaced hidden scrollbar with thin themed scrollbar</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>index.css</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Code Quality</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>PDF base64 encoding optimized</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Replaced manual char-by-char loop with Array.from + join</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>pdfGen.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Branding</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>aiq_ prefix renamed to cma_</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Changed localStorage keys from aiq_ to cma_ prefix</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>store.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Branding</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>App ID changed</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>com.accountiq.app -&gt; com.cmacompass.app</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>capacitor.config.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Branding</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>DB connection renamed</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>accountiq -&gt; cmacompass in db.ts and pdfGen.ts</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>db.ts, pdfGen.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>README project structure fixed</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Added missing PaperScreen.tsx and LevelScreen.tsx references</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>README.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>CI: SHA-256 hash asset added</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Added sha256sum step and web-build.zip.sha256 to release assets</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>build-apk.yml</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Audit</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Full Security &amp; Quality Audit</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>All 21 issues fixed: 5 Critical, 7 Medium, 4 Low. TS + Vite build pass. Brain log updated.</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>21 files changed</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Reconnect phone via ADB wireless</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Wireless debugging disconnected. User needs to re-enable and provide new IP:port.</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Install v2.5.2 APK on phone</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>APK built at android/app/build/outputs/apk/debug/app-debug.apk. Waiting for ADB connection.</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Git commit all changes</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Stage and commit the 21 fixes for v2.5.2.</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Push to GitHub main</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Push commit to trigger CI build + release.</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Create GitHub release v2.5.2</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Ensure release shows as Latest on GitHub with APK + web-build.zip + sha256 assets.</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>20-07-2026</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Update Excel brain log</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Log v2.5.2 release with all changes and deployment status.</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>